<commit_message>
added scenario to fail the testcase in excel sheet
</commit_message>
<xml_diff>
--- a/Test1/SOC_TestCase.xlsx
+++ b/Test1/SOC_TestCase.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="8360" activeTab="2"/>
+    <workbookView windowWidth="19200" windowHeight="8000"/>
   </bookViews>
   <sheets>
     <sheet name="TC_0001" sheetId="8" r:id="rId1"/>
@@ -1244,7 +1244,7 @@
         <v>50</v>
       </c>
       <c r="H6" s="4">
-        <v>49.997</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" ht="16.5" spans="1:8">

</xml_diff>